<commit_message>
did some part 3 stuff, right now starting regression
</commit_message>
<xml_diff>
--- a/Interviews_Survey/Interview_Analysis.xlsx
+++ b/Interviews_Survey/Interview_Analysis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Studium\X_Masterarbeit\Data\Master_Thesis\Interviews_Survey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B87B8A-EFB9-4248-B58E-12F39F7EFDDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F20EC0CB-01F0-4869-8519-736CB30FA656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -153,9 +153,6 @@
     <t>Promotion strategy</t>
   </si>
   <si>
-    <t>You never know what will work. You need to find the one person that will become a super user</t>
-  </si>
-  <si>
     <t>There's no clear answer to what works and what does not because luck is involved</t>
   </si>
   <si>
@@ -415,6 +412,9 @@
   </si>
   <si>
     <t>Overall Topic Nr</t>
+  </si>
+  <si>
+    <t>You never know what will work. You need to find the one person that will become a superuser</t>
   </si>
 </sst>
 </file>
@@ -533,22 +533,22 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -856,7 +856,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -865,7 +865,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -881,8 +881,8 @@
       <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="8" t="s">
-        <v>123</v>
+      <c r="F2" s="11" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -898,7 +898,7 @@
       <c r="D3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="8"/>
+      <c r="F3" s="11"/>
     </row>
     <row r="4" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
@@ -913,7 +913,7 @@
       <c r="D4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="8"/>
+      <c r="F4" s="11"/>
     </row>
     <row r="5" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -931,8 +931,8 @@
       <c r="E5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>124</v>
+      <c r="F5" s="8" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -951,7 +951,7 @@
       <c r="E6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="7"/>
+      <c r="F6" s="8"/>
     </row>
     <row r="7" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
@@ -969,7 +969,7 @@
       <c r="E7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="7"/>
+      <c r="F7" s="8"/>
     </row>
     <row r="8" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -987,7 +987,7 @@
       <c r="E8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="7"/>
+      <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
@@ -1005,7 +1005,7 @@
       <c r="E9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="7"/>
+      <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
@@ -1023,7 +1023,7 @@
       <c r="E10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="7"/>
+      <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
@@ -1041,7 +1041,7 @@
       <c r="E11" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F11" s="7"/>
+      <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
@@ -1059,7 +1059,7 @@
       <c r="E12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F12" s="7"/>
+      <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
@@ -1074,8 +1074,8 @@
       <c r="D13" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="10" t="s">
-        <v>126</v>
+      <c r="F13" s="12" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -1091,7 +1091,7 @@
       <c r="D14" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F14" s="10"/>
+      <c r="F14" s="12"/>
     </row>
     <row r="15" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
@@ -1106,7 +1106,7 @@
       <c r="D15" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F15" s="10"/>
+      <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
@@ -1121,7 +1121,7 @@
       <c r="D16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F16" s="10"/>
+      <c r="F16" s="12"/>
     </row>
     <row r="17" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
@@ -1136,7 +1136,7 @@
       <c r="D17" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F17" s="10"/>
+      <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
@@ -1154,7 +1154,7 @@
       <c r="E18" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F18" s="10"/>
+      <c r="F18" s="12"/>
     </row>
     <row r="19" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
@@ -1170,10 +1170,10 @@
         <v>24</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1205,7 +1205,7 @@
         <v>26</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F21" s="9"/>
     </row>
@@ -1223,7 +1223,7 @@
         <v>27</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F22" s="9"/>
     </row>
@@ -1241,7 +1241,7 @@
         <v>28</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F23" s="9"/>
     </row>
@@ -1292,7 +1292,7 @@
         <v>2</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F26" s="9"/>
     </row>
@@ -1337,10 +1337,10 @@
         <v>3</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>124</v>
+        <v>129</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="30" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1354,9 +1354,9 @@
         <v>3</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F30" s="7"/>
+        <v>42</v>
+      </c>
+      <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
@@ -1369,12 +1369,12 @@
         <v>3</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F31" s="7"/>
+        <v>50</v>
+      </c>
+      <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
@@ -1387,12 +1387,12 @@
         <v>3</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F32" s="7"/>
+        <v>50</v>
+      </c>
+      <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
@@ -1405,12 +1405,12 @@
         <v>3</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F33" s="7"/>
+        <v>51</v>
+      </c>
+      <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
@@ -1423,12 +1423,12 @@
         <v>3</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F34" s="7"/>
+        <v>46</v>
+      </c>
+      <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
@@ -1441,12 +1441,12 @@
         <v>3</v>
       </c>
       <c r="D35" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E35" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F35" s="7"/>
+      <c r="F35" s="8"/>
     </row>
     <row r="36" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
@@ -1459,9 +1459,9 @@
         <v>3</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="F36" s="7"/>
+        <v>52</v>
+      </c>
+      <c r="F36" s="8"/>
     </row>
     <row r="37" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
@@ -1474,12 +1474,12 @@
         <v>3</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F37" s="7"/>
+        <v>50</v>
+      </c>
+      <c r="F37" s="8"/>
     </row>
     <row r="38" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
@@ -1492,28 +1492,28 @@
         <v>3</v>
       </c>
       <c r="D38" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E38" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E38" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F38" s="7"/>
+      <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C39" s="5">
+        <v>4</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C39" s="5">
-        <v>4</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>124</v>
+      <c r="F39" s="8" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="40" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1521,67 +1521,67 @@
         <v>4</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C40" s="5">
         <v>4</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F40" s="7"/>
+        <v>66</v>
+      </c>
+      <c r="F40" s="8"/>
     </row>
     <row r="41" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C41" s="6">
         <v>4</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F41" s="7"/>
+        <v>59</v>
+      </c>
+      <c r="F41" s="8"/>
     </row>
     <row r="42" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C42" s="6">
         <v>4</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="F42" s="7"/>
+        <v>66</v>
+      </c>
+      <c r="F42" s="8"/>
     </row>
     <row r="43" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C43" s="5">
+        <v>4</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C43" s="5">
-        <v>4</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>124</v>
+      <c r="F43" s="8" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="44" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1589,151 +1589,151 @@
         <v>4</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C44" s="5">
         <v>4</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F44" s="7"/>
+        <v>72</v>
+      </c>
+      <c r="F44" s="8"/>
     </row>
     <row r="45" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C45" s="5">
         <v>4</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F45" s="7"/>
+        <v>63</v>
+      </c>
+      <c r="F45" s="8"/>
     </row>
     <row r="46" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C46" s="5">
         <v>4</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="F46" s="7"/>
+        <v>117</v>
+      </c>
+      <c r="F46" s="8"/>
     </row>
     <row r="47" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C47" s="5">
         <v>4</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="F47" s="7"/>
+        <v>65</v>
+      </c>
+      <c r="F47" s="8"/>
     </row>
     <row r="48" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C48" s="6">
         <v>4</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F48" s="7"/>
+        <v>68</v>
+      </c>
+      <c r="F48" s="8"/>
     </row>
     <row r="49" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C49" s="6">
         <v>4</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="F49" s="7"/>
+        <v>69</v>
+      </c>
+      <c r="F49" s="8"/>
     </row>
     <row r="50" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C50" s="6">
         <v>4</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F50" s="7"/>
+        <v>50</v>
+      </c>
+      <c r="F50" s="8"/>
     </row>
     <row r="51" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C51" s="6">
         <v>4</v>
       </c>
       <c r="D51" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E51" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="E51" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F51" s="7"/>
+      <c r="F51" s="8"/>
     </row>
     <row r="52" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C52" s="5">
         <v>3</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>22</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="53" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -1741,16 +1741,16 @@
         <v>6</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C53" s="6">
         <v>3</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F53" s="9"/>
     </row>
@@ -1759,13 +1759,13 @@
         <v>6</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C54" s="6">
         <v>3</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F54" s="9"/>
     </row>
@@ -1774,13 +1774,13 @@
         <v>6</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C55" s="6">
         <v>3</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F55" s="9"/>
     </row>
@@ -1789,16 +1789,16 @@
         <v>6</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C56" s="6">
         <v>3</v>
       </c>
       <c r="D56" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E56" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>80</v>
       </c>
       <c r="F56" s="9"/>
     </row>
@@ -1807,13 +1807,13 @@
         <v>6</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C57" s="6">
         <v>3</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F57" s="9"/>
     </row>
@@ -1822,16 +1822,16 @@
         <v>4</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C58" s="5">
         <v>5</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F58" s="12" t="s">
-        <v>127</v>
+        <v>82</v>
+      </c>
+      <c r="F58" s="10" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="59" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1839,154 +1839,154 @@
         <v>4</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C59" s="5">
         <v>5</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F59" s="12"/>
+        <v>88</v>
+      </c>
+      <c r="F59" s="10"/>
     </row>
     <row r="60" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C60" s="5">
         <v>5</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F60" s="12"/>
+        <v>83</v>
+      </c>
+      <c r="F60" s="10"/>
     </row>
     <row r="61" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C61" s="5">
         <v>5</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F61" s="12"/>
+        <v>84</v>
+      </c>
+      <c r="F61" s="10"/>
     </row>
     <row r="62" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C62" s="5">
         <v>5</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="F62" s="12"/>
+        <v>85</v>
+      </c>
+      <c r="F62" s="10"/>
     </row>
     <row r="63" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C63" s="5">
         <v>5</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F63" s="12"/>
+        <v>105</v>
+      </c>
+      <c r="F63" s="10"/>
     </row>
     <row r="64" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C64" s="5">
         <v>5</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F64" s="12"/>
+        <v>87</v>
+      </c>
+      <c r="F64" s="10"/>
     </row>
     <row r="65" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C65" s="6">
         <v>5</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F65" s="12"/>
+        <v>46</v>
+      </c>
+      <c r="F65" s="10"/>
     </row>
     <row r="66" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C66" s="6">
         <v>5</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F66" s="12"/>
+        <v>107</v>
+      </c>
+      <c r="F66" s="10"/>
     </row>
     <row r="67" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C67" s="6">
         <v>5</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="F67" s="12"/>
+        <v>90</v>
+      </c>
+      <c r="F67" s="10"/>
     </row>
     <row r="68" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C68" s="5">
         <v>5</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="69" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1994,13 +1994,13 @@
         <v>4</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C69" s="5">
         <v>5</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F69" s="9"/>
     </row>
@@ -2009,13 +2009,13 @@
         <v>6</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C70" s="6">
         <v>5</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F70" s="9"/>
     </row>
@@ -2024,16 +2024,16 @@
         <v>4</v>
       </c>
       <c r="B71" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C71" s="5">
+        <v>4</v>
+      </c>
+      <c r="D71" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C71" s="5">
-        <v>4</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="F71" s="7" t="s">
-        <v>124</v>
+      <c r="F71" s="8" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="72" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -2041,76 +2041,76 @@
         <v>4</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C72" s="5">
         <v>4</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F72" s="7"/>
+        <v>97</v>
+      </c>
+      <c r="F72" s="8"/>
     </row>
     <row r="73" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C73" s="5">
         <v>4</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="F73" s="7"/>
+        <v>98</v>
+      </c>
+      <c r="F73" s="8"/>
     </row>
     <row r="74" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C74" s="6">
         <v>4</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="F74" s="7"/>
+        <v>99</v>
+      </c>
+      <c r="F74" s="8"/>
     </row>
     <row r="75" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C75" s="6">
         <v>4</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="F75" s="7"/>
+        <v>100</v>
+      </c>
+      <c r="F75" s="8"/>
     </row>
     <row r="76" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B76" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C76" s="5">
+        <v>4</v>
+      </c>
+      <c r="D76" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C76" s="5">
-        <v>4</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F76" s="11" t="s">
-        <v>128</v>
+      <c r="F76" s="7" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="77" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -2118,76 +2118,76 @@
         <v>4</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C77" s="5">
         <v>4</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F77" s="11"/>
+        <v>103</v>
+      </c>
+      <c r="F77" s="7"/>
     </row>
     <row r="78" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C78" s="5">
         <v>4</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F78" s="11"/>
+        <v>104</v>
+      </c>
+      <c r="F78" s="7"/>
     </row>
     <row r="79" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A79" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C79" s="6">
         <v>4</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="F79" s="11"/>
+        <v>118</v>
+      </c>
+      <c r="F79" s="7"/>
     </row>
     <row r="80" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A80" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C80" s="6">
         <v>4</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="F80" s="11"/>
+        <v>106</v>
+      </c>
+      <c r="F80" s="7"/>
     </row>
     <row r="81" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C81" s="5">
         <v>6</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F81" s="7" t="s">
-        <v>124</v>
+        <v>108</v>
+      </c>
+      <c r="F81" s="8" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="82" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -2195,61 +2195,61 @@
         <v>4</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C82" s="5">
         <v>6</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="F82" s="7"/>
+        <v>109</v>
+      </c>
+      <c r="F82" s="8"/>
     </row>
     <row r="83" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C83" s="6">
         <v>6</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="F83" s="7"/>
+        <v>110</v>
+      </c>
+      <c r="F83" s="8"/>
     </row>
     <row r="84" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C84" s="6">
         <v>6</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="F84" s="7"/>
+        <v>111</v>
+      </c>
+      <c r="F84" s="8"/>
     </row>
     <row r="85" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B85" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C85" s="5">
+        <v>6</v>
+      </c>
+      <c r="D85" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C85" s="5">
-        <v>6</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>114</v>
-      </c>
       <c r="F85" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="86" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -2257,13 +2257,13 @@
         <v>4</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C86" s="5">
         <v>6</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F86" s="9"/>
     </row>
@@ -2272,13 +2272,13 @@
         <v>4</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C87" s="5">
         <v>6</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F87" s="9"/>
     </row>
@@ -2287,18 +2287,24 @@
         <v>6</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C88" s="6">
         <v>6</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F88" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="F39:F42"/>
+    <mergeCell ref="F2:F4"/>
+    <mergeCell ref="F5:F12"/>
+    <mergeCell ref="F19:F28"/>
+    <mergeCell ref="F13:F18"/>
+    <mergeCell ref="F29:F38"/>
     <mergeCell ref="F76:F80"/>
     <mergeCell ref="F81:F84"/>
     <mergeCell ref="F85:F88"/>
@@ -2307,12 +2313,6 @@
     <mergeCell ref="F58:F67"/>
     <mergeCell ref="F68:F70"/>
     <mergeCell ref="F71:F75"/>
-    <mergeCell ref="F39:F42"/>
-    <mergeCell ref="F2:F4"/>
-    <mergeCell ref="F5:F12"/>
-    <mergeCell ref="F19:F28"/>
-    <mergeCell ref="F13:F18"/>
-    <mergeCell ref="F29:F38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>